<commit_message>
fix svm baseline to predict new format of data
</commit_message>
<xml_diff>
--- a/GenData/events_gt_df.xlsx
+++ b/GenData/events_gt_df.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="7">
   <si>
     <t xml:space="preserve">time_start</t>
   </si>
@@ -31,16 +31,16 @@
     <t xml:space="preserve">eID</t>
   </si>
   <si>
+    <t xml:space="preserve">eID_2</t>
+  </si>
+  <si>
     <t xml:space="preserve">eID_5</t>
   </si>
   <si>
-    <t xml:space="preserve">eID_2</t>
+    <t xml:space="preserve">eID_1</t>
   </si>
   <si>
     <t xml:space="preserve">eID_4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eID_1</t>
   </si>
 </sst>
 </file>
@@ -53,7 +53,7 @@
   <fonts count="4">
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -116,16 +116,8 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -142,9 +134,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="LibreOffice">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
@@ -152,46 +144,46 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="18A303"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="0369A3"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A33E03"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8E03A3"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="C99C00"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="C9211E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000EE"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="551A8B"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme>
@@ -199,25 +191,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter/>
         </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter/>
         </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:prstDash val="solid"/>
-          <a:miter/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -235,12 +260,48 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
+        </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
@@ -252,101 +313,215 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="0" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="0" t="n">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>99.95</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="B2" s="0" t="n">
+        <v>49.05</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>53.85</v>
+      </c>
+      <c r="D2" s="0" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>153.65</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>153.7</v>
-      </c>
-      <c r="D3" s="1" t="s">
+      <c r="B3" s="0" t="n">
+        <v>79.3</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="D3" s="0" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="0" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="n">
+      <c r="B4" s="0" t="n">
+        <v>129.35</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>131.75</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>152.8</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>157.4</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>171.2</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>172.75</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>182.85</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>183.75</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>196.6</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>199.95</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>214.45</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>215.4</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>243.65</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>246.9</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="0" t="n">
         <v>247.4</v>
       </c>
-      <c r="C4" s="1" t="n">
+      <c r="C11" s="0" t="n">
         <v>248.15</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D11" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>253.3</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>254.4</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>267.1</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>271.65</v>
+      </c>
+      <c r="D13" s="0" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>277.1</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>283.65</v>
+      </c>
+      <c r="D14" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>277.55</v>
-      </c>
-      <c r="C5" s="1" t="n">
-        <v>278.15</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>297.1</v>
-      </c>
-      <c r="C6" s="1" t="n">
-        <v>297.45</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>294.6</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>299.95</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
start reworking k-fold cross validation
</commit_message>
<xml_diff>
--- a/GenData/events_gt_df.xlsx
+++ b/GenData/events_gt_df.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -435,153 +435,153 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>7.9</v>
+        <v>5</v>
       </c>
       <c r="B2" t="n">
-        <v>46.45</v>
+        <v>75.25</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>48.9</v>
+        <v>79.3</v>
       </c>
       <c r="B3" t="n">
-        <v>55.3</v>
+        <v>102.5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>61.85</v>
+        <v>129.35</v>
       </c>
       <c r="B4" t="n">
-        <v>125.55</v>
+        <v>131.75</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>129.35</v>
+        <v>171.2</v>
       </c>
       <c r="B5" t="n">
-        <v>129.7</v>
+        <v>172.75</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>129.7</v>
+        <v>182.85</v>
       </c>
       <c r="B6" t="n">
-        <v>129.7</v>
+        <v>183.75</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>129.75</v>
+        <v>196.6</v>
       </c>
       <c r="B7" t="n">
-        <v>129.75</v>
+        <v>199.95</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>129.75</v>
+        <v>214.45</v>
       </c>
       <c r="B8" t="n">
-        <v>129.75</v>
+        <v>215.4</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>129.8</v>
+        <v>217</v>
       </c>
       <c r="B9" t="n">
-        <v>129.8</v>
+        <v>217.9</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>129.8</v>
+        <v>243.65</v>
       </c>
       <c r="B10" t="n">
-        <v>129.8</v>
+        <v>246.9</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>129.85</v>
+        <v>252</v>
       </c>
       <c r="B11" t="n">
-        <v>129.85</v>
+        <v>253.3</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>129.85</v>
+        <v>254.35</v>
       </c>
       <c r="B12" t="n">
-        <v>129.9</v>
+        <v>254.4</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>129.9</v>
+        <v>267.1</v>
       </c>
       <c r="B13" t="n">
-        <v>129.95</v>
+        <v>271.65</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -591,10 +591,10 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>129.95</v>
+        <v>278.05</v>
       </c>
       <c r="B14" t="n">
-        <v>129.95</v>
+        <v>284.75</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -604,49 +604,49 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>130</v>
+        <v>287.2</v>
       </c>
       <c r="B15" t="n">
-        <v>130</v>
+        <v>290.15</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>130</v>
+        <v>294.6</v>
       </c>
       <c r="B16" t="n">
-        <v>130</v>
+        <v>297.25</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>130.05</v>
+        <v>334.85</v>
       </c>
       <c r="B17" t="n">
-        <v>131.75</v>
+        <v>336.35</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>152.45</v>
+        <v>352.15</v>
       </c>
       <c r="B18" t="n">
-        <v>157.65</v>
+        <v>352.55</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -656,49 +656,49 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>170.3</v>
+        <v>354.55</v>
       </c>
       <c r="B19" t="n">
-        <v>174</v>
+        <v>356.1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>182.85</v>
+        <v>375.25</v>
       </c>
       <c r="B20" t="n">
-        <v>183.75</v>
+        <v>389.4</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>eID_1</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>194.95</v>
+        <v>397.95</v>
       </c>
       <c r="B21" t="n">
-        <v>201</v>
+        <v>403.35</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>214.45</v>
+        <v>407.75</v>
       </c>
       <c r="B22" t="n">
-        <v>215.4</v>
+        <v>407.9</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -708,62 +708,62 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>220.45</v>
+        <v>417.2</v>
       </c>
       <c r="B23" t="n">
-        <v>247.4</v>
+        <v>447</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>247.4</v>
+        <v>466.15</v>
       </c>
       <c r="B24" t="n">
-        <v>247.4</v>
+        <v>470.35</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>eID_4</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>247.45</v>
+        <v>472.3</v>
       </c>
       <c r="B25" t="n">
-        <v>247.85</v>
+        <v>478.6</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>247.85</v>
+        <v>484.9</v>
       </c>
       <c r="B26" t="n">
-        <v>247.85</v>
+        <v>486.5</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>eID_4</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>247.9</v>
+        <v>493.45</v>
       </c>
       <c r="B27" t="n">
-        <v>247.95</v>
+        <v>496.4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -773,36 +773,36 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>248</v>
+        <v>505.85</v>
       </c>
       <c r="B28" t="n">
-        <v>248.15</v>
+        <v>549.45</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>eID_4</t>
+          <t>eID_2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>251.9</v>
+        <v>552.15</v>
       </c>
       <c r="B29" t="n">
-        <v>256.3</v>
+        <v>556.3</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>eID_5</t>
+          <t>eID_1</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>267.1</v>
+        <v>557.3</v>
       </c>
       <c r="B30" t="n">
-        <v>271.65</v>
+        <v>557.3</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -812,27 +812,1574 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>276.95</v>
+        <v>563.55</v>
       </c>
       <c r="B31" t="n">
-        <v>283.8</v>
+        <v>575.25</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>eID_2</t>
+          <t>eID_5</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>294.6</v>
+        <v>578.95</v>
       </c>
       <c r="B32" t="n">
-        <v>299.95</v>
+        <v>582.1</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
           <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>611.25</v>
+      </c>
+      <c r="B33" t="n">
+        <v>613.9</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>625.55</v>
+      </c>
+      <c r="B34" t="n">
+        <v>629.9</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>648.8</v>
+      </c>
+      <c r="B35" t="n">
+        <v>652.25</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>677.4</v>
+      </c>
+      <c r="B36" t="n">
+        <v>679.3</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>690.25</v>
+      </c>
+      <c r="B37" t="n">
+        <v>693.6</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>708.2</v>
+      </c>
+      <c r="B38" t="n">
+        <v>709.55</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>730.55</v>
+      </c>
+      <c r="B39" t="n">
+        <v>732.3</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>797.7</v>
+      </c>
+      <c r="B40" t="n">
+        <v>821.95</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>847.15</v>
+      </c>
+      <c r="B41" t="n">
+        <v>909.8</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>912.9</v>
+      </c>
+      <c r="B42" t="n">
+        <v>913.4</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>932.55</v>
+      </c>
+      <c r="B43" t="n">
+        <v>933.6</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>937.3</v>
+      </c>
+      <c r="B44" t="n">
+        <v>937.75</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>945.15</v>
+      </c>
+      <c r="B45" t="n">
+        <v>991.4</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>994.35</v>
+      </c>
+      <c r="B46" t="n">
+        <v>995.75</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>998.05</v>
+      </c>
+      <c r="B47" t="n">
+        <v>998.05</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>999.05</v>
+      </c>
+      <c r="B48" t="n">
+        <v>999.1</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1001.3</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1001.35</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>1002.35</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1002.35</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1035.6</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1037.95</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>1058.45</v>
+      </c>
+      <c r="B52" t="n">
+        <v>1154.3</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1198.95</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1199.05</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>1203.75</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1205.6</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>1208.4</v>
+      </c>
+      <c r="B55" t="n">
+        <v>1213.05</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>1227.8</v>
+      </c>
+      <c r="B56" t="n">
+        <v>1228.4</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>1240.1</v>
+      </c>
+      <c r="B57" t="n">
+        <v>1241.45</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>1255.65</v>
+      </c>
+      <c r="B58" t="n">
+        <v>1257.75</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>1274.45</v>
+      </c>
+      <c r="B59" t="n">
+        <v>1275.8</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>1278.25</v>
+      </c>
+      <c r="B60" t="n">
+        <v>1322.9</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>1327.55</v>
+      </c>
+      <c r="B61" t="n">
+        <v>1329.1</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>1346.5</v>
+      </c>
+      <c r="B62" t="n">
+        <v>1351.3</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>1372.7</v>
+      </c>
+      <c r="B63" t="n">
+        <v>1377.65</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>1404.85</v>
+      </c>
+      <c r="B64" t="n">
+        <v>1408.7</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>1411.55</v>
+      </c>
+      <c r="B65" t="n">
+        <v>1413.65</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>1441.05</v>
+      </c>
+      <c r="B66" t="n">
+        <v>1443.1</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>1445.9</v>
+      </c>
+      <c r="B67" t="n">
+        <v>1451.1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>1459</v>
+      </c>
+      <c r="B68" t="n">
+        <v>1460.4</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>1470.9</v>
+      </c>
+      <c r="B69" t="n">
+        <v>1471.1</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>1478.2</v>
+      </c>
+      <c r="B70" t="n">
+        <v>1478.2</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>1493.8</v>
+      </c>
+      <c r="B71" t="n">
+        <v>1497.3</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>1498.3</v>
+      </c>
+      <c r="B72" t="n">
+        <v>1498.3</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>1504.45</v>
+      </c>
+      <c r="B73" t="n">
+        <v>1547.2</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>1563.2</v>
+      </c>
+      <c r="B74" t="n">
+        <v>1576.1</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>1592.25</v>
+      </c>
+      <c r="B75" t="n">
+        <v>1593.8</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>1596.95</v>
+      </c>
+      <c r="B76" t="n">
+        <v>1601.7</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>1619.2</v>
+      </c>
+      <c r="B77" t="n">
+        <v>1621</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>1627.1</v>
+      </c>
+      <c r="B78" t="n">
+        <v>1642.75</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>1651.3</v>
+      </c>
+      <c r="B79" t="n">
+        <v>1658.55</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>1793.35</v>
+      </c>
+      <c r="B80" t="n">
+        <v>1820.95</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>1835.5</v>
+      </c>
+      <c r="B81" t="n">
+        <v>1836.85</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>1838.75</v>
+      </c>
+      <c r="B82" t="n">
+        <v>1839.3</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>1879.7</v>
+      </c>
+      <c r="B83" t="n">
+        <v>1928.75</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>1933.1</v>
+      </c>
+      <c r="B84" t="n">
+        <v>1936.85</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>1997.85</v>
+      </c>
+      <c r="B85" t="n">
+        <v>1998.35</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>2001.45</v>
+      </c>
+      <c r="B86" t="n">
+        <v>2006.55</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>2013.85</v>
+      </c>
+      <c r="B87" t="n">
+        <v>2014.95</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>2015.95</v>
+      </c>
+      <c r="B88" t="n">
+        <v>2015.95</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>2016.95</v>
+      </c>
+      <c r="B89" t="n">
+        <v>2018.45</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>2059.8</v>
+      </c>
+      <c r="B90" t="n">
+        <v>2060.8</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>2079.75</v>
+      </c>
+      <c r="B91" t="n">
+        <v>2087.7</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>2095.8</v>
+      </c>
+      <c r="B92" t="n">
+        <v>2096</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>2097.75</v>
+      </c>
+      <c r="B93" t="n">
+        <v>2101.75</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>2105</v>
+      </c>
+      <c r="B94" t="n">
+        <v>2124.5</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>2159.9</v>
+      </c>
+      <c r="B95" t="n">
+        <v>2165.7</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>2173.2</v>
+      </c>
+      <c r="B96" t="n">
+        <v>2173.85</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>2184.7</v>
+      </c>
+      <c r="B97" t="n">
+        <v>2185.3</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>2226.85</v>
+      </c>
+      <c r="B98" t="n">
+        <v>2255.1</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>2259.5</v>
+      </c>
+      <c r="B99" t="n">
+        <v>2259.95</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>2269.85</v>
+      </c>
+      <c r="B100" t="n">
+        <v>2273.1</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>2279.2</v>
+      </c>
+      <c r="B101" t="n">
+        <v>2282.55</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>2302.8</v>
+      </c>
+      <c r="B102" t="n">
+        <v>2370.5</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>2375.85</v>
+      </c>
+      <c r="B103" t="n">
+        <v>2393</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>2403.9</v>
+      </c>
+      <c r="B104" t="n">
+        <v>2405.75</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>2433.1</v>
+      </c>
+      <c r="B105" t="n">
+        <v>2434.65</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>2464.5</v>
+      </c>
+      <c r="B106" t="n">
+        <v>2464.55</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>2496.45</v>
+      </c>
+      <c r="B107" t="n">
+        <v>2496.45</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>2499.4</v>
+      </c>
+      <c r="B108" t="n">
+        <v>2500.55</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>2505</v>
+      </c>
+      <c r="B109" t="n">
+        <v>2514.9</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>2523.6</v>
+      </c>
+      <c r="B110" t="n">
+        <v>2526.65</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>2543.05</v>
+      </c>
+      <c r="B111" t="n">
+        <v>2544.2</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>2568.45</v>
+      </c>
+      <c r="B112" t="n">
+        <v>2569.6</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>2582.5</v>
+      </c>
+      <c r="B113" t="n">
+        <v>2583.5</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>2594.9</v>
+      </c>
+      <c r="B114" t="n">
+        <v>2595.95</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>2626</v>
+      </c>
+      <c r="B115" t="n">
+        <v>2629.9</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>2638</v>
+      </c>
+      <c r="B116" t="n">
+        <v>2640.45</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>2671.3</v>
+      </c>
+      <c r="B117" t="n">
+        <v>2676.6</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>2686.7</v>
+      </c>
+      <c r="B118" t="n">
+        <v>2688.3</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>2696.75</v>
+      </c>
+      <c r="B119" t="n">
+        <v>2700.85</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>2708.25</v>
+      </c>
+      <c r="B120" t="n">
+        <v>2709.05</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>2717.35</v>
+      </c>
+      <c r="B121" t="n">
+        <v>2717.85</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>2737.15</v>
+      </c>
+      <c r="B122" t="n">
+        <v>2737.15</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>2764.45</v>
+      </c>
+      <c r="B123" t="n">
+        <v>2766.75</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>2777.7</v>
+      </c>
+      <c r="B124" t="n">
+        <v>2783.1</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>2807.8</v>
+      </c>
+      <c r="B125" t="n">
+        <v>2848.75</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>2861.5</v>
+      </c>
+      <c r="B126" t="n">
+        <v>2863.25</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>2875.8</v>
+      </c>
+      <c r="B127" t="n">
+        <v>2879.95</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>2880.95</v>
+      </c>
+      <c r="B128" t="n">
+        <v>2883.9</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>2894.55</v>
+      </c>
+      <c r="B129" t="n">
+        <v>2896.1</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>2963.05</v>
+      </c>
+      <c r="B130" t="n">
+        <v>2966</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>2992.9</v>
+      </c>
+      <c r="B131" t="n">
+        <v>2994.35</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>3016.85</v>
+      </c>
+      <c r="B132" t="n">
+        <v>3021.7</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>3053.25</v>
+      </c>
+      <c r="B133" t="n">
+        <v>3069.95</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>3086.25</v>
+      </c>
+      <c r="B134" t="n">
+        <v>3096.15</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>3108.85</v>
+      </c>
+      <c r="B135" t="n">
+        <v>3113.25</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>3142.15</v>
+      </c>
+      <c r="B136" t="n">
+        <v>3168.55</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>3177.85</v>
+      </c>
+      <c r="B137" t="n">
+        <v>3179.2</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>3192.45</v>
+      </c>
+      <c r="B138" t="n">
+        <v>3194.4</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>3198.7</v>
+      </c>
+      <c r="B139" t="n">
+        <v>3199.9</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>3202.85</v>
+      </c>
+      <c r="B140" t="n">
+        <v>3205.2</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>3220.95</v>
+      </c>
+      <c r="B141" t="n">
+        <v>3222.15</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>3227.8</v>
+      </c>
+      <c r="B142" t="n">
+        <v>3250.4</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>3260.05</v>
+      </c>
+      <c r="B143" t="n">
+        <v>3263.15</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>3270.2</v>
+      </c>
+      <c r="B144" t="n">
+        <v>3270.4</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>3333.15</v>
+      </c>
+      <c r="B145" t="n">
+        <v>3338</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>3359.8</v>
+      </c>
+      <c r="B146" t="n">
+        <v>3359.8</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>3377.5</v>
+      </c>
+      <c r="B147" t="n">
+        <v>3381.15</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>eID_3</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>3389.35</v>
+      </c>
+      <c r="B148" t="n">
+        <v>3405.75</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>eID_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>3424.5</v>
+      </c>
+      <c r="B149" t="n">
+        <v>3545.45</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>eID_5</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>3550.7</v>
+      </c>
+      <c r="B150" t="n">
+        <v>3553.75</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>eID_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>3556.7</v>
+      </c>
+      <c r="B151" t="n">
+        <v>3586.6</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>eID_3</t>
         </is>
       </c>
     </row>

</xml_diff>